<commit_message>
feat: inventaire postes avec 12 membres Claude Code (licences Teams)
- Onglet "Inventaire Postes" rempli avec les 12 membres actifs
- 7 Premium (Developer), 4 Standard, 1 Unassigned
- Colonnes: Nom, Email, Role, Licence, Profil Deploy, Poste, CC Version, etc.
- Copie des docs vers le dossier Teams sync pour partage via SharePoint

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runbook-Deploiement-ClaudeCode-CAGM.xlsx
+++ b/Runbook-Deploiement-ClaudeCode-CAGM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist Deploiement" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Inventaire Postes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Configuration" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Acces Reseau" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist Deploiement" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventaire Postes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acces Reseau" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,8 +71,14 @@
       <color rgb="001F4E79"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +115,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -163,6 +174,27 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2229,20 +2261,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2253,59 +2287,554 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Licence</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Profil Deploy</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Utilisateur</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Profil</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Date deploy.</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Claude Code</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>CC Version</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>Desktop</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>VS Code Ext.</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Plugin</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
         <is>
           <t>CShip</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Win Terminal</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>Status Deploy</t>
+        </is>
+      </c>
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>Date Deploy</t>
+        </is>
+      </c>
+      <c r="M3" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Melissa</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>m.benkadoum@gmining.com</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="21" t="n"/>
+      <c r="H4" s="21" t="n"/>
+      <c r="I4" s="21" t="n"/>
+      <c r="J4" s="21" t="n"/>
+      <c r="K4" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L4" s="21" t="n"/>
+      <c r="M4" s="21" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Jonathan</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>j.gingras@gmining.com</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
+      <c r="I5" s="21" t="n"/>
+      <c r="J5" s="21" t="n"/>
+      <c r="K5" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="n"/>
+      <c r="M5" s="21" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Philippe</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>p.lanthier@gmining.com</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="21" t="n"/>
+      <c r="J6" s="21" t="n"/>
+      <c r="K6" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L6" s="21" t="n"/>
+      <c r="M6" s="21" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>j.lalonde@gmining.com</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="21" t="n"/>
+      <c r="H7" s="21" t="n"/>
+      <c r="I7" s="21" t="n"/>
+      <c r="J7" s="21" t="n"/>
+      <c r="K7" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L7" s="21" t="n"/>
+      <c r="M7" s="21" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Julie</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>j.blouin@gmining.com</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="n"/>
+      <c r="G8" s="21" t="n"/>
+      <c r="H8" s="21" t="n"/>
+      <c r="I8" s="21" t="n"/>
+      <c r="J8" s="21" t="n"/>
+      <c r="K8" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L8" s="21" t="n"/>
+      <c r="M8" s="21" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Sebastien Gagnon</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>s.gagnon@gmining.com</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L9" s="21" t="n"/>
+      <c r="M9" s="21" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Mathieu</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>m.rheaume@gmining.com</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="21" t="n"/>
+      <c r="I10" s="21" t="n"/>
+      <c r="J10" s="21" t="n"/>
+      <c r="K10" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L10" s="21" t="n"/>
+      <c r="M10" s="21" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>a.deslauriers@gmining.com</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="21" t="n"/>
+      <c r="I11" s="21" t="n"/>
+      <c r="J11" s="21" t="n"/>
+      <c r="K11" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L11" s="21" t="n"/>
+      <c r="M11" s="21" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>administrator@gmining.com</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>Primary Owner</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="21" t="n"/>
+      <c r="J12" s="21" t="n"/>
+      <c r="K12" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L12" s="21" t="n"/>
+      <c r="M12" s="21" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Giselle</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>g.mendes@gmining.com</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="21" t="n"/>
+      <c r="I13" s="21" t="n"/>
+      <c r="J13" s="21" t="n"/>
+      <c r="K13" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="n"/>
+      <c r="M13" s="21" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Xime</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>x.benavides@gmining.com</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="21" t="n"/>
+      <c r="I14" s="21" t="n"/>
+      <c r="J14" s="21" t="n"/>
+      <c r="K14" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L14" s="21" t="n"/>
+      <c r="M14" s="21" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>s.gabriel@gmining.com</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="24" t="inlineStr">
+        <is>
+          <t>A deployer</t>
+        </is>
+      </c>
+      <c r="L15" s="21" t="n"/>
+      <c r="M15" s="21" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>12 membres</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>7 Premium / 4 Standard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: statuts deploiement par membre dans Inventaire Postes
- Sebastien: Deploye (full stack Developer)
- Jeremy: Partiel (VS Code OK, Cowork a deployer)
- Melissa, Philippe, Jonathan: Partiel (Cowork OK, Standard)
- Julie, Mathieu, Giselle, Xime, SG: A deployer (Cowork)
- Alex: A confirmer
- Anthony: Admin (Unassigned)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Runbook-Deploiement-ClaudeCode-CAGM.xlsx
+++ b/Runbook-Deploiement-ClaudeCode-CAGM.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +76,26 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C6500"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="9">
@@ -138,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -196,6 +216,25 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2261,7 +2300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2376,21 +2415,29 @@
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="F4" s="21" t="n"/>
-      <c r="G4" s="21" t="n"/>
-      <c r="H4" s="21" t="n"/>
-      <c r="I4" s="21" t="n"/>
-      <c r="J4" s="21" t="n"/>
-      <c r="K4" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L4" s="21" t="n"/>
-      <c r="M4" s="21" t="n"/>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr"/>
+      <c r="G4" s="21" t="inlineStr"/>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>Cowork OK</t>
+        </is>
+      </c>
+      <c r="I4" s="21" t="inlineStr"/>
+      <c r="J4" s="21" t="inlineStr"/>
+      <c r="K4" s="27" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="L4" s="21" t="inlineStr"/>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>Cowork OK. WSL non deploye (Standard = pas requis).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2415,21 +2462,29 @@
       </c>
       <c r="E5" s="23" t="inlineStr">
         <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="F5" s="21" t="n"/>
-      <c r="G5" s="21" t="n"/>
-      <c r="H5" s="21" t="n"/>
-      <c r="I5" s="21" t="n"/>
-      <c r="J5" s="21" t="n"/>
-      <c r="K5" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L5" s="21" t="n"/>
-      <c r="M5" s="21" t="n"/>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr"/>
+      <c r="G5" s="21" t="inlineStr"/>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>Cowork OK</t>
+        </is>
+      </c>
+      <c r="I5" s="21" t="inlineStr"/>
+      <c r="J5" s="21" t="inlineStr"/>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="inlineStr"/>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>Cowork OK. WSL non deploye (Standard = pas requis).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2454,21 +2509,29 @@
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="F6" s="21" t="n"/>
-      <c r="G6" s="21" t="n"/>
-      <c r="H6" s="21" t="n"/>
-      <c r="I6" s="21" t="n"/>
-      <c r="J6" s="21" t="n"/>
-      <c r="K6" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L6" s="21" t="n"/>
-      <c r="M6" s="21" t="n"/>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr"/>
+      <c r="G6" s="21" t="inlineStr"/>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>Cowork OK</t>
+        </is>
+      </c>
+      <c r="I6" s="21" t="inlineStr"/>
+      <c r="J6" s="21" t="inlineStr"/>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="L6" s="21" t="inlineStr"/>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>Cowork OK. WSL non deploye (Standard = pas requis).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2496,18 +2559,26 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="F7" s="21" t="n"/>
-      <c r="G7" s="21" t="n"/>
-      <c r="H7" s="21" t="n"/>
-      <c r="I7" s="21" t="n"/>
-      <c r="J7" s="21" t="n"/>
-      <c r="K7" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L7" s="21" t="n"/>
-      <c r="M7" s="21" t="n"/>
+      <c r="F7" s="21" t="inlineStr"/>
+      <c r="G7" s="21" t="inlineStr"/>
+      <c r="H7" s="21" t="inlineStr">
+        <is>
+          <t>VS Code OK</t>
+        </is>
+      </c>
+      <c r="I7" s="21" t="inlineStr"/>
+      <c r="J7" s="21" t="inlineStr"/>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="L7" s="21" t="inlineStr"/>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>VS Code fonctionne. Cowork a deployer.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2532,21 +2603,25 @@
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="21" t="n"/>
-      <c r="H8" s="21" t="n"/>
-      <c r="I8" s="21" t="n"/>
-      <c r="J8" s="21" t="n"/>
-      <c r="K8" s="24" t="inlineStr">
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr"/>
+      <c r="G8" s="21" t="inlineStr"/>
+      <c r="H8" s="21" t="inlineStr"/>
+      <c r="I8" s="21" t="inlineStr"/>
+      <c r="J8" s="21" t="inlineStr"/>
+      <c r="K8" s="28" t="inlineStr">
         <is>
           <t>A deployer</t>
         </is>
       </c>
-      <c r="L8" s="21" t="n"/>
-      <c r="M8" s="21" t="n"/>
+      <c r="L8" s="21" t="inlineStr"/>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>Cowork a deployer</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2574,18 +2649,46 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="F9" s="21" t="n"/>
-      <c r="G9" s="21" t="n"/>
-      <c r="H9" s="21" t="n"/>
-      <c r="I9" s="21" t="n"/>
-      <c r="J9" s="21" t="n"/>
-      <c r="K9" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L9" s="21" t="n"/>
-      <c r="M9" s="21" t="n"/>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>BN69594</t>
+        </is>
+      </c>
+      <c r="G9" s="21" t="inlineStr">
+        <is>
+          <t>2.1.97</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" s="21" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="K9" s="29" t="inlineStr">
+        <is>
+          <t>Deploye</t>
+        </is>
+      </c>
+      <c r="L9" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>Full stack: CC + Desktop + Cowork + WSL + VS Code + ATLAS + CShip</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2613,18 +2716,22 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="F10" s="21" t="n"/>
-      <c r="G10" s="21" t="n"/>
-      <c r="H10" s="21" t="n"/>
-      <c r="I10" s="21" t="n"/>
-      <c r="J10" s="21" t="n"/>
-      <c r="K10" s="24" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr"/>
+      <c r="G10" s="21" t="inlineStr"/>
+      <c r="H10" s="21" t="inlineStr"/>
+      <c r="I10" s="21" t="inlineStr"/>
+      <c r="J10" s="21" t="inlineStr"/>
+      <c r="K10" s="28" t="inlineStr">
         <is>
           <t>A deployer</t>
         </is>
       </c>
-      <c r="L10" s="21" t="n"/>
-      <c r="M10" s="21" t="n"/>
+      <c r="L10" s="21" t="inlineStr"/>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>Cowork a deployer</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2652,18 +2759,22 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="F11" s="21" t="n"/>
-      <c r="G11" s="21" t="n"/>
-      <c r="H11" s="21" t="n"/>
-      <c r="I11" s="21" t="n"/>
-      <c r="J11" s="21" t="n"/>
-      <c r="K11" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L11" s="21" t="n"/>
-      <c r="M11" s="21" t="n"/>
+      <c r="F11" s="21" t="inlineStr"/>
+      <c r="G11" s="21" t="inlineStr"/>
+      <c r="H11" s="21" t="inlineStr"/>
+      <c r="I11" s="21" t="inlineStr"/>
+      <c r="J11" s="21" t="inlineStr"/>
+      <c r="K11" s="30" t="inlineStr">
+        <is>
+          <t>A confirmer</t>
+        </is>
+      </c>
+      <c r="L11" s="21" t="inlineStr"/>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>Confirmer avec Alex avant deploiement</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2691,18 +2802,22 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="21" t="n"/>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="24" t="inlineStr">
-        <is>
-          <t>A deployer</t>
-        </is>
-      </c>
-      <c r="L12" s="21" t="n"/>
-      <c r="M12" s="21" t="n"/>
+      <c r="F12" s="21" t="inlineStr"/>
+      <c r="G12" s="21" t="inlineStr"/>
+      <c r="H12" s="21" t="inlineStr"/>
+      <c r="I12" s="21" t="inlineStr"/>
+      <c r="J12" s="21" t="inlineStr"/>
+      <c r="K12" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="21" t="inlineStr"/>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>Compte admin — licence Unassigned</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2730,18 +2845,22 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="21" t="n"/>
-      <c r="H13" s="21" t="n"/>
-      <c r="I13" s="21" t="n"/>
-      <c r="J13" s="21" t="n"/>
-      <c r="K13" s="24" t="inlineStr">
+      <c r="F13" s="21" t="inlineStr"/>
+      <c r="G13" s="21" t="inlineStr"/>
+      <c r="H13" s="21" t="inlineStr"/>
+      <c r="I13" s="21" t="inlineStr"/>
+      <c r="J13" s="21" t="inlineStr"/>
+      <c r="K13" s="28" t="inlineStr">
         <is>
           <t>A deployer</t>
         </is>
       </c>
-      <c r="L13" s="21" t="n"/>
-      <c r="M13" s="21" t="n"/>
+      <c r="L13" s="21" t="inlineStr"/>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>Cowork a deployer</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2769,18 +2888,22 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="21" t="n"/>
-      <c r="H14" s="21" t="n"/>
-      <c r="I14" s="21" t="n"/>
-      <c r="J14" s="21" t="n"/>
-      <c r="K14" s="24" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr"/>
+      <c r="G14" s="21" t="inlineStr"/>
+      <c r="H14" s="21" t="inlineStr"/>
+      <c r="I14" s="21" t="inlineStr"/>
+      <c r="J14" s="21" t="inlineStr"/>
+      <c r="K14" s="28" t="inlineStr">
         <is>
           <t>A deployer</t>
         </is>
       </c>
-      <c r="L14" s="21" t="n"/>
-      <c r="M14" s="21" t="n"/>
+      <c r="L14" s="21" t="inlineStr"/>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>Cowork a deployer</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2808,18 +2931,22 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="21" t="n"/>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="21" t="n"/>
-      <c r="J15" s="21" t="n"/>
-      <c r="K15" s="24" t="inlineStr">
+      <c r="F15" s="21" t="inlineStr"/>
+      <c r="G15" s="21" t="inlineStr"/>
+      <c r="H15" s="21" t="inlineStr"/>
+      <c r="I15" s="21" t="inlineStr"/>
+      <c r="J15" s="21" t="inlineStr"/>
+      <c r="K15" s="28" t="inlineStr">
         <is>
           <t>A deployer</t>
         </is>
       </c>
-      <c r="L15" s="21" t="n"/>
-      <c r="M15" s="21" t="n"/>
+      <c r="L15" s="21" t="inlineStr"/>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t>S. Gabriel — Developer profile</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2835,6 +2962,32 @@
       <c r="D17" s="16" t="inlineStr">
         <is>
           <t>7 Premium / 4 Standard</t>
+        </is>
+      </c>
+      <c r="K17" s="32" t="inlineStr">
+        <is>
+          <t>Deploye: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="K18" s="33" t="inlineStr">
+        <is>
+          <t>Partiel: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="K19" s="34" t="inlineStr">
+        <is>
+          <t>A deployer: 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="K20" s="35" t="inlineStr">
+        <is>
+          <t>A confirmer: 1</t>
         </is>
       </c>
     </row>

</xml_diff>